<commit_message>
Auto-opdater EPGOAL 2026-10-07 16:44:59
</commit_message>
<xml_diff>
--- a/reports/variant_groups_v3.xlsx
+++ b/reports/variant_groups_v3.xlsx
@@ -14,11 +14,11 @@
     <sheet name="TV3-TV3plus" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Variant Groups'!$A$1:$L$62</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stream Details'!$A$1:$J$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Problems'!$A$1:$J$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TV3-TV3plus'!$A$1:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stream Details'!$A$1:$J$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Problems'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TV3-TV3plus'!$A$1:$J$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,11 +62,6 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4B084"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -80,14 +75,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -480,7 +474,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06 15:41:40</t>
+          <t>2026-10-07 15:25:10</t>
         </is>
       </c>
     </row>
@@ -523,13 +517,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Streamstatus: FORKERT KANAL</t>
+          <t>Streamstatus: MANGLER EPG</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -539,35 +533,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Streamstatus: MANGLER EPG</t>
+          <t>Streamstatus: MANGLER TVG-ID</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Streamstatus: MANGLER TVG-ID</t>
+          <t>Streamstatus: OK</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Streamstatus: OK</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -674,7 +658,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
@@ -722,7 +706,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
@@ -770,7 +754,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>243</v>
+        <v>226</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -814,7 +798,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
@@ -986,7 +970,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="E9" t="n">
         <v>6</v>
@@ -1034,7 +1018,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
@@ -1126,7 +1110,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
@@ -1218,7 +1202,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E14" t="n">
         <v>4</v>
@@ -1310,7 +1294,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
@@ -1358,7 +1342,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
@@ -1406,7 +1390,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
@@ -1454,7 +1438,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="E19" t="n">
         <v>4</v>
@@ -1502,7 +1486,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E20" t="n">
         <v>5</v>
@@ -1550,7 +1534,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>
@@ -1598,7 +1582,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E22" t="n">
         <v>3</v>
@@ -1646,7 +1630,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E23" t="n">
         <v>3</v>
@@ -1766,7 +1750,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E26" t="n">
         <v>4</v>
@@ -1862,7 +1846,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E28" t="n">
         <v>6</v>
@@ -1946,7 +1930,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E30" t="n">
         <v>5</v>
@@ -1994,7 +1978,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E31" t="n">
         <v>2</v>
@@ -2110,7 +2094,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E34" t="n">
         <v>2</v>
@@ -2234,7 +2218,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
@@ -2274,7 +2258,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -2314,7 +2298,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E39" t="n">
         <v>6</v>
@@ -2362,7 +2346,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
@@ -2406,7 +2390,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E41" t="n">
         <v>3</v>
@@ -2494,7 +2478,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E43" t="n">
         <v>3</v>
@@ -2542,7 +2526,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E44" t="n">
         <v>2</v>
@@ -2590,7 +2574,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E45" t="n">
         <v>3</v>
@@ -2638,7 +2622,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E46" t="n">
         <v>3</v>
@@ -2686,7 +2670,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E47" t="n">
         <v>3</v>
@@ -2734,7 +2718,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="E48" t="n">
         <v>3</v>
@@ -2782,7 +2766,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="E49" t="n">
         <v>3</v>
@@ -2830,7 +2814,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E50" t="n">
         <v>3</v>
@@ -2881,10 +2865,10 @@
         <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G51" t="n">
         <v>1</v>
@@ -2900,60 +2884,60 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
+          <t>tv3.dk x3</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>TV3 DK [Denmark], TV3 FHD DK [Denmark], TV3 HD DK [Denmark]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>175</v>
+      </c>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>1</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
           <t>tv3plus.dk x3</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>TV3 DK [Denmark], TV3 FHD DK [Denmark], TV3 HD DK [Denmark], TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>180</v>
-      </c>
-      <c r="E52" t="n">
-        <v>6</v>
-      </c>
-      <c r="F52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G52" t="n">
-        <v>2</v>
-      </c>
-      <c r="H52" t="n">
-        <v>2</v>
-      </c>
-      <c r="I52" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" t="n">
-        <v>1</v>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>tv3plus.dk x3</t>
-        </is>
-      </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>TV3 DK [Denmark], TV3 FHD DK [Denmark], TV3 HD DK [Denmark], TV3+ DK [Denmark], TV3+ FHD DK [Denmark], TV3+ HD DK [Denmark]</t>
+          <t>TV3+ DK [Denmark], TV3+ FHD DK [Denmark], TV3+ HD DK [Denmark]</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3158,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="E58" t="n">
         <v>2</v>
@@ -3262,7 +3246,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E60" t="n">
         <v>1</v>
@@ -3354,7 +3338,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E62" t="n">
         <v>2</v>
@@ -3397,11 +3381,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="41" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="53" customWidth="1" min="5" max="5"/>
@@ -3497,7 +3481,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -3506,7 +3490,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>EPGShare:6'eren.dk(97); BSS:6eren.dk(52); OpenEPG:6'eren.dk(146)</t>
+          <t>EPGShare:6'eren.dk(91); BSS:6eren.dk(52); OpenEPG:6'eren.dk(146)</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3527,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3552,7 +3536,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>EPGShare:6'eren.dk(97); BSS:6eren.dk(52); OpenEPG:6'eren.dk(146)</t>
+          <t>EPGShare:6'eren.dk(91); BSS:6eren.dk(52); OpenEPG:6'eren.dk(146)</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3573,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -3598,7 +3582,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>EPGShare:6'eren.dk(97); BSS:6eren.dk(52); OpenEPG:6'eren.dk(146)</t>
+          <t>EPGShare:6'eren.dk(91); BSS:6eren.dk(52); OpenEPG:6'eren.dk(146)</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3619,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -3644,7 +3628,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>EPGShare:Animal.Planet.dk(111); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
+          <t>EPGShare:Animal.Planet.dk(113); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3665,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3690,7 +3674,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>EPGShare:Animal.Planet.dk(111); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
+          <t>EPGShare:Animal.Planet.dk(113); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3711,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3736,7 +3720,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>EPGShare:Animal.Planet.dk(111); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
+          <t>EPGShare:Animal.Planet.dk(113); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3761,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3823,7 +3807,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3832,7 +3816,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>EPGShare:Animal.Planet.dk(111); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
+          <t>EPGShare:Animal.Planet.dk(113); BSS:animalplanet.dk(54); OpenEPG:Animal Planet.dk(174)</t>
         </is>
       </c>
     </row>
@@ -3873,7 +3857,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>243</v>
+        <v>226</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3919,7 +3903,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3928,7 +3912,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>EPGShare:BBC.Nordic.dk(141); BSS:bbcnordic.dk(72); OpenEPG:BBC NORDIC.dk(149)</t>
+          <t>EPGShare:BBC.Nordic.dk(140); BSS:bbcnordic.dk(72); OpenEPG:BBC NORDIC.dk(149)</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3949,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3974,7 +3958,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>EPGShare:BBC.Nordic.dk(141); BSS:bbcnordic.dk(72); OpenEPG:BBC NORDIC.dk(149)</t>
+          <t>EPGShare:BBC.Nordic.dk(140); BSS:bbcnordic.dk(72); OpenEPG:BBC NORDIC.dk(149)</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4042,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>EPGShare:Canal.9.dk(94); BSS:canal9.dk(47); OpenEPG:canal9.dk(51)</t>
+          <t>EPGShare:Canal.9.dk(94); BSS:canal9.dk(47); OpenEPG:Canal9.dk(98)</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4088,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>EPGShare:Canal.9.dk(94); BSS:canal9.dk(47); OpenEPG:canal9.dk(51)</t>
+          <t>EPGShare:Canal.9.dk(94); BSS:canal9.dk(47); OpenEPG:Canal9.dk(98)</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4134,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>EPGShare:Canal.9.dk(94); BSS:canal9.dk(47); OpenEPG:canal9.dk(51)</t>
+          <t>EPGShare:Canal.9.dk(94); BSS:canal9.dk(47); OpenEPG:Canal9.dk(98)</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4171,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4196,7 +4180,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoon.Network.dk(493); BSS:cartoonnetwork.dk(240); OpenEPG:cartoonnetwork.dk(252)</t>
+          <t>EPGShare:Cartoon.Network.dk(489); BSS:cartoonnetwork.dk(240); OpenEPG:Cartoon Network.dk(742)</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4217,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4242,7 +4226,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoon.Network.dk(493); BSS:cartoonnetwork.dk(240); OpenEPG:cartoonnetwork.dk(252)</t>
+          <t>EPGShare:Cartoon.Network.dk(489); BSS:cartoonnetwork.dk(240); OpenEPG:Cartoon Network.dk(742)</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4263,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4288,7 +4272,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoon.Network.dk(493); BSS:cartoonnetwork.dk(240); OpenEPG:cartoonnetwork.dk(252)</t>
+          <t>EPGShare:Cartoon.Network.dk(489); BSS:cartoonnetwork.dk(240); OpenEPG:Cartoon Network.dk(742)</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4309,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4334,7 +4318,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoon.Network.dk(493); BSS:cartoonnetwork.dk(240); OpenEPG:cartoonnetwork.dk(252)</t>
+          <t>EPGShare:Cartoon.Network.dk(489); BSS:cartoonnetwork.dk(240); OpenEPG:Cartoon Network.dk(742)</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4355,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4380,7 +4364,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoon.Network.dk(493); BSS:cartoonnetwork.dk(240); OpenEPG:cartoonnetwork.dk(252)</t>
+          <t>EPGShare:Cartoon.Network.dk(489); BSS:cartoonnetwork.dk(240); OpenEPG:Cartoon Network.dk(742)</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4405,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4467,7 +4451,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4476,7 +4460,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoonito.dk(593); BSS:cartoonito.dk(292); OpenEPG:Cartoonito.dk(605)</t>
+          <t>EPGShare:Cartoonito.dk(589); BSS:cartoonito.dk(292); OpenEPG:Cartoonito.dk(605)</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4497,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4522,7 +4506,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoonito.dk(593); BSS:cartoonito.dk(292); OpenEPG:Cartoonito.dk(605)</t>
+          <t>EPGShare:Cartoonito.dk(589); BSS:cartoonito.dk(292); OpenEPG:Cartoonito.dk(605)</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4543,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4568,7 +4552,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>EPGShare:Cartoonito.dk(593); BSS:cartoonito.dk(292); OpenEPG:Cartoonito.dk(605)</t>
+          <t>EPGShare:Cartoonito.dk(589); BSS:cartoonito.dk(292); OpenEPG:Cartoonito.dk(605)</t>
         </is>
       </c>
     </row>
@@ -4789,7 +4773,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4798,7 +4782,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>EPGShare:Discovery.Channel.dk(95); BSS:discoverychannel.dk(46); OpenEPG:discoverychannel.dk(0)</t>
+          <t>EPGShare:Discovery.Channel.dk(94); BSS:discoverychannel.dk(46); OpenEPG:Discovery Channel.dk(138)</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4819,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -4844,7 +4828,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>EPGShare:Discovery.Channel.dk(95); BSS:discoverychannel.dk(46); OpenEPG:discoverychannel.dk(0)</t>
+          <t>EPGShare:Discovery.Channel.dk(94); BSS:discoverychannel.dk(46); OpenEPG:Discovery Channel.dk(138)</t>
         </is>
       </c>
     </row>
@@ -4885,7 +4869,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -4940,7 +4924,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>EPGShare:Discovery.Science.dk(4); BSS:discoveryscience.dk(2); OpenEPG:discoveryscience.dk(82)</t>
+          <t>EPGShare:Discovery.Science.dk(4); BSS:discoveryscience.dk(2); OpenEPG:Discovery Science.dk(236)</t>
         </is>
       </c>
     </row>
@@ -4977,7 +4961,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -4986,7 +4970,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>EPGShare:Disney.Channel.dk(215); BSS:disneychannel.dk(118); OpenEPG:Disney Channel.dk(138)</t>
+          <t>EPGShare:Disney.Channel.dk(213); BSS:disneychannel.dk(118); OpenEPG:disneychannel.dk(113)</t>
         </is>
       </c>
     </row>
@@ -5023,7 +5007,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -5032,7 +5016,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>EPGShare:Disney.Channel.dk(215); BSS:disneychannel.dk(118); OpenEPG:Disney Channel.dk(138)</t>
+          <t>EPGShare:Disney.Channel.dk(213); BSS:disneychannel.dk(118); OpenEPG:disneychannel.dk(113)</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5057,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -5119,7 +5103,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -5128,7 +5112,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>EPGShare:Disney.Channel.dk(215); BSS:disneychannel.dk(118); OpenEPG:Disney Channel.dk(138)</t>
+          <t>EPGShare:Disney.Channel.dk(213); BSS:disneychannel.dk(118); OpenEPG:disneychannel.dk(113)</t>
         </is>
       </c>
     </row>
@@ -5303,7 +5287,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -5312,7 +5296,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>EPGShare:DR.Ramasjang.dk(309); BSS:drramasjang.dk(150); OpenEPG:DR Ramasjang.dk(505)</t>
+          <t>EPGShare:DR.Ramasjang.dk(302); BSS:drramasjang.dk(150); OpenEPG:DR Ramasjang.dk(505)</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5333,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -5358,7 +5342,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>EPGShare:DR.Ramasjang.dk(309); BSS:drramasjang.dk(150); OpenEPG:DR Ramasjang.dk(505)</t>
+          <t>EPGShare:DR.Ramasjang.dk(302); BSS:drramasjang.dk(150); OpenEPG:DR Ramasjang.dk(505)</t>
         </is>
       </c>
     </row>
@@ -5395,7 +5379,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -5404,7 +5388,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>EPGShare:DR1.dk(128); BSS:dr1.dk(62); OpenEPG:DR1.dk(195)</t>
+          <t>EPGShare:DR1.dk(132); BSS:dr1.dk(62); OpenEPG:dr1.dk(66)</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5425,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -5450,7 +5434,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>EPGShare:DR1.dk(128); BSS:dr1.dk(62); OpenEPG:DR1.dk(195)</t>
+          <t>EPGShare:DR1.dk(132); BSS:dr1.dk(62); OpenEPG:dr1.dk(66)</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5471,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -5496,7 +5480,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>EPGShare:DR1.dk(128); BSS:dr1.dk(62); OpenEPG:DR1.dk(195)</t>
+          <t>EPGShare:DR1.dk(132); BSS:dr1.dk(62); OpenEPG:dr1.dk(66)</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5517,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -5542,7 +5526,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>EPGShare:DR2.dk(107); BSS:dr2.dk(55); OpenEPG:DR2.dk(148)</t>
+          <t>EPGShare:DR2.dk(104); BSS:dr2.dk(55); OpenEPG:DR2.dk(148)</t>
         </is>
       </c>
     </row>
@@ -5579,7 +5563,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -5588,7 +5572,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>EPGShare:DR2.dk(107); BSS:dr2.dk(55); OpenEPG:DR2.dk(148)</t>
+          <t>EPGShare:DR2.dk(104); BSS:dr2.dk(55); OpenEPG:DR2.dk(148)</t>
         </is>
       </c>
     </row>
@@ -5625,7 +5609,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -5634,7 +5618,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>EPGShare:DR2.dk(107); BSS:dr2.dk(55); OpenEPG:DR2.dk(148)</t>
+          <t>EPGShare:DR2.dk(104); BSS:dr2.dk(55); OpenEPG:DR2.dk(148)</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5655,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -5680,7 +5664,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.1.dk(72); BSS:eurosport1.dk(29); OpenEPG:Eurosport 1.dk(87)</t>
+          <t>EPGShare:Eurosport.1.dk(66); BSS:eurosport1.dk(29); OpenEPG:Eurosport 1.dk(87)</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5701,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -5726,7 +5710,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.1.dk(72); BSS:eurosport1.dk(29); OpenEPG:Eurosport 1.dk(87)</t>
+          <t>EPGShare:Eurosport.1.dk(66); BSS:eurosport1.dk(29); OpenEPG:Eurosport 1.dk(87)</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5751,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -5813,7 +5797,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -5822,7 +5806,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.1.dk(72); BSS:eurosport1.dk(29); OpenEPG:Eurosport 1.dk(87)</t>
+          <t>EPGShare:Eurosport.1.dk(66); BSS:eurosport1.dk(29); OpenEPG:Eurosport 1.dk(87)</t>
         </is>
       </c>
     </row>
@@ -5859,7 +5843,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -5868,7 +5852,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.2.dk(66); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
+          <t>EPGShare:Eurosport.2.dk(64); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
         </is>
       </c>
     </row>
@@ -5905,7 +5889,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -5914,7 +5898,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.2.dk(66); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
+          <t>EPGShare:Eurosport.2.dk(64); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5935,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -5960,7 +5944,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.2.dk(66); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
+          <t>EPGShare:Eurosport.2.dk(64); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
         </is>
       </c>
     </row>
@@ -6001,7 +5985,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -6047,7 +6031,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -6056,7 +6040,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>EPGShare:Eurosport.2.dk(66); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
+          <t>EPGShare:Eurosport.2.dk(64); BSS:eurosport2.dk(44); OpenEPG:eurosport2.dk(31)</t>
         </is>
       </c>
     </row>
@@ -6093,7 +6077,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -6102,7 +6086,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>EPGShare:Investigation.Discovery.dk(104); BSS:investigationdiscovery.dk(51); OpenEPG:Investigation Discovery.dk(100)</t>
+          <t>EPGShare:Investigation.Discovery.dk(102); BSS:investigationdiscovery.dk(51); OpenEPG:Investigation Discovery.dk(100)</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6123,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -6148,7 +6132,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>EPGShare:Investigation.Discovery.dk(104); BSS:investigationdiscovery.dk(51); OpenEPG:Investigation Discovery.dk(100)</t>
+          <t>EPGShare:Investigation.Discovery.dk(102); BSS:investigationdiscovery.dk(51); OpenEPG:Investigation Discovery.dk(100)</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6169,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -6194,7 +6178,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>EPGShare:Investigation.Discovery.dk(104); BSS:investigationdiscovery.dk(51); OpenEPG:Investigation Discovery.dk(100)</t>
+          <t>EPGShare:Investigation.Discovery.dk(102); BSS:investigationdiscovery.dk(51); OpenEPG:Investigation Discovery.dk(100)</t>
         </is>
       </c>
     </row>
@@ -6231,7 +6215,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -6240,7 +6224,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>EPGShare:Kanal.4.dk(121); BSS:kanal4.dk(56); OpenEPG:kanal4.dk(57)</t>
+          <t>EPGShare:Kanal.4.dk(118); BSS:kanal4.dk(56); OpenEPG:Kanal 4.dk(167)</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6261,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -6286,7 +6270,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>EPGShare:Kanal.4.dk(121); BSS:kanal4.dk(56); OpenEPG:kanal4.dk(57)</t>
+          <t>EPGShare:Kanal.4.dk(118); BSS:kanal4.dk(56); OpenEPG:Kanal 4.dk(167)</t>
         </is>
       </c>
     </row>
@@ -6323,7 +6307,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -6332,7 +6316,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>EPGShare:Kanal.4.dk(121); BSS:kanal4.dk(56); OpenEPG:kanal4.dk(57)</t>
+          <t>EPGShare:Kanal.4.dk(118); BSS:kanal4.dk(56); OpenEPG:Kanal 4.dk(167)</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6353,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -6378,7 +6362,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>EPGShare:Kanal.5.dk(102); BSS:kanal5.dk(51); OpenEPG:Kanal 5.dk(140)</t>
+          <t>EPGShare:Kanal.5.dk(99); BSS:kanal5.dk(51); OpenEPG:Kanal 5.dk(140)</t>
         </is>
       </c>
     </row>
@@ -6415,7 +6399,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -6424,7 +6408,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>EPGShare:Kanal.5.dk(102); BSS:kanal5.dk(51); OpenEPG:Kanal 5.dk(140)</t>
+          <t>EPGShare:Kanal.5.dk(99); BSS:kanal5.dk(51); OpenEPG:Kanal 5.dk(140)</t>
         </is>
       </c>
     </row>
@@ -6461,7 +6445,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
@@ -6470,7 +6454,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>EPGShare:Kanal.5.dk(102); BSS:kanal5.dk(51); OpenEPG:Kanal 5.dk(140)</t>
+          <t>EPGShare:Kanal.5.dk(99); BSS:kanal5.dk(51); OpenEPG:Kanal 5.dk(140)</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6495,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
@@ -6561,7 +6545,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
@@ -6611,7 +6595,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
@@ -6661,7 +6645,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -6716,7 +6700,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:National Geographic.dk(49)</t>
+          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:nationalgeographic.dk(54)</t>
         </is>
       </c>
     </row>
@@ -6762,7 +6746,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:National Geographic.dk(49)</t>
+          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:nationalgeographic.dk(54)</t>
         </is>
       </c>
     </row>
@@ -6808,7 +6792,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:National Geographic.dk(49)</t>
+          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:nationalgeographic.dk(54)</t>
         </is>
       </c>
     </row>
@@ -6854,7 +6838,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:National Geographic.dk(49)</t>
+          <t>EPGShare:National.Geographic.dk(97); BSS:nationalgeographic.dk(48); OpenEPG:nationalgeographic.dk(54)</t>
         </is>
       </c>
     </row>
@@ -6891,7 +6875,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -6900,7 +6884,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>EPGShare:Nick.Jr..dk(300); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
+          <t>EPGShare:Nick.Jr..dk(299); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
         </is>
       </c>
     </row>
@@ -6937,7 +6921,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -6946,7 +6930,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>EPGShare:Nick.Jr..dk(300); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
+          <t>EPGShare:Nick.Jr..dk(299); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
         </is>
       </c>
     </row>
@@ -6983,7 +6967,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
@@ -6992,7 +6976,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>EPGShare:Nick.Jr..dk(300); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
+          <t>EPGShare:Nick.Jr..dk(299); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7013,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
@@ -7038,7 +7022,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>EPGShare:Nick.Jr..dk(300); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
+          <t>EPGShare:Nick.Jr..dk(299); BSS:nickjr.dk(178); OpenEPG:Nick Jr.dk(160)</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7063,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
@@ -7088,7 +7072,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>BSS:Nick Jr.(0)</t>
+          <t>BSS:nick_jr(0)</t>
         </is>
       </c>
     </row>
@@ -7129,7 +7113,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -7138,7 +7122,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>BSS:Nick Jr.(0)</t>
+          <t>BSS:nick_jr(0)</t>
         </is>
       </c>
     </row>
@@ -7175,7 +7159,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -7184,7 +7168,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>EPGShare:Nickelodeon.dk(245); BSS:nickelodeon.dk(127); OpenEPG:Nickelodeon.dk(514)</t>
+          <t>EPGShare:Nickelodeon.dk(246); BSS:nickelodeon.dk(127); OpenEPG:nickelodeon.dk(132)</t>
         </is>
       </c>
     </row>
@@ -7221,7 +7205,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -7230,7 +7214,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>EPGShare:Nickelodeon.dk(245); BSS:nickelodeon.dk(127); OpenEPG:Nickelodeon.dk(514)</t>
+          <t>EPGShare:Nickelodeon.dk(246); BSS:nickelodeon.dk(127); OpenEPG:nickelodeon.dk(132)</t>
         </is>
       </c>
     </row>
@@ -7267,7 +7251,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -7276,7 +7260,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>EPGShare:Nickelodeon.dk(245); BSS:nickelodeon.dk(127); OpenEPG:Nickelodeon.dk(514)</t>
+          <t>EPGShare:Nickelodeon.dk(246); BSS:nickelodeon.dk(127); OpenEPG:nickelodeon.dk(132)</t>
         </is>
       </c>
     </row>
@@ -7313,7 +7297,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -7322,7 +7306,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>EPGShare:Nickelodeon.dk(245); BSS:nickelodeon.dk(127); OpenEPG:Nickelodeon.dk(514)</t>
+          <t>EPGShare:Nickelodeon.dk(246); BSS:nickelodeon.dk(127); OpenEPG:nickelodeon.dk(132)</t>
         </is>
       </c>
     </row>
@@ -7363,7 +7347,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
@@ -7413,7 +7397,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
@@ -7463,7 +7447,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
@@ -7509,7 +7493,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -7518,7 +7502,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>EPGShare:See.dk(148); BSS:see.dk(67); OpenEPG:See.dk(274)</t>
+          <t>EPGShare:See.dk(144); BSS:see.dk(67); OpenEPG:See.dk(274)</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7539,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -7564,7 +7548,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>EPGShare:See.dk(148); BSS:see.dk(67); OpenEPG:See.dk(274)</t>
+          <t>EPGShare:See.dk(144); BSS:see.dk(67); OpenEPG:See.dk(274)</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7594,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>BSS:sfkanalen.dk(2); OpenEPG:SF-kanalen.dk(30)</t>
+          <t>BSS:sfkanalen.dk(2); OpenEPG:sfkanalen.dk(32)</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7631,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -7656,7 +7640,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>EPGShare:TLC.dk(86); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
+          <t>EPGShare:TLC.dk(89); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
         </is>
       </c>
     </row>
@@ -7693,7 +7677,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -7702,7 +7686,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>EPGShare:TLC.dk(86); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
+          <t>EPGShare:TLC.dk(89); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
         </is>
       </c>
     </row>
@@ -7739,7 +7723,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -7748,7 +7732,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>EPGShare:TLC.dk(86); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
+          <t>EPGShare:TLC.dk(89); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
         </is>
       </c>
     </row>
@@ -7785,7 +7769,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -7794,7 +7778,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>EPGShare:TLC.dk(86); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
+          <t>EPGShare:TLC.dk(89); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
         </is>
       </c>
     </row>
@@ -7835,7 +7819,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -7881,7 +7865,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
@@ -7890,7 +7874,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>EPGShare:TLC.dk(86); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
+          <t>EPGShare:TLC.dk(89); BSS:tlc.dk(41); OpenEPG:tlc.dk(47)</t>
         </is>
       </c>
     </row>
@@ -7927,7 +7911,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
@@ -7973,7 +7957,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -7982,7 +7966,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Fri.dk(124); BSS:tv2fri.dk(64); OpenEPG:TV 2 Fri.dk(127)</t>
+          <t>EPGShare:TV.2.Fri.dk(123); BSS:tv2fri.dk(64); OpenEPG:TV2 FRI.dk(61)</t>
         </is>
       </c>
     </row>
@@ -8019,7 +8003,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
@@ -8028,7 +8012,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Fri.dk(124); BSS:tv2fri.dk(64); OpenEPG:TV 2 Fri.dk(127)</t>
+          <t>EPGShare:TV.2.Fri.dk(123); BSS:tv2fri.dk(64); OpenEPG:TV2 FRI.dk(61)</t>
         </is>
       </c>
     </row>
@@ -8065,7 +8049,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
@@ -8074,7 +8058,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Fri.dk(124); BSS:tv2fri.dk(64); OpenEPG:TV 2 Fri.dk(127)</t>
+          <t>EPGShare:TV.2.Fri.dk(123); BSS:tv2fri.dk(64); OpenEPG:TV2 FRI.dk(61)</t>
         </is>
       </c>
     </row>
@@ -8115,7 +8099,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
@@ -8124,7 +8108,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.News.dk(58); BSS:tv2news.dk(30); OpenEPG:TV 2 News.dk(55)</t>
+          <t>EPGShare:TV.2.News.dk(55); BSS:tv2news.dk(30); OpenEPG:tv2news.dk(27)</t>
         </is>
       </c>
     </row>
@@ -8165,7 +8149,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
@@ -8174,7 +8158,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.News.dk(58); BSS:tv2news.dk(30); OpenEPG:TV 2 News.dk(55)</t>
+          <t>EPGShare:TV.2.News.dk(55); BSS:tv2news.dk(30); OpenEPG:tv2news.dk(27)</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8199,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
@@ -8224,7 +8208,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.News.dk(58); BSS:tv2news.dk(30); OpenEPG:TV 2 News.dk(55)</t>
+          <t>EPGShare:TV.2.News.dk(55); BSS:tv2news.dk(30); OpenEPG:tv2news.dk(27)</t>
         </is>
       </c>
     </row>
@@ -8261,7 +8245,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
@@ -8270,7 +8254,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Sport.X.dk(57); BSS:tv2sportx.dk(54); OpenEPG:tv2sportx.dk(54)</t>
+          <t>EPGShare:TV.2.Sport.X.dk(46); BSS:tv2sportx.dk(54); OpenEPG:TV2 Sport X.dk(48)</t>
         </is>
       </c>
     </row>
@@ -8307,7 +8291,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
@@ -8316,7 +8300,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Sport.X.dk(57); BSS:tv2sportx.dk(54); OpenEPG:tv2sportx.dk(54)</t>
+          <t>EPGShare:TV.2.Sport.X.dk(46); BSS:tv2sportx.dk(54); OpenEPG:TV2 Sport X.dk(48)</t>
         </is>
       </c>
     </row>
@@ -8353,7 +8337,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -8362,7 +8346,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.dk(121); BSS:tv2.dk(58); OpenEPG:TV2.dk(51)</t>
+          <t>EPGShare:TV.2.dk(115); BSS:tv2.dk(58); OpenEPG:TV 2.dk(57)</t>
         </is>
       </c>
     </row>
@@ -8399,7 +8383,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
@@ -8408,7 +8392,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.dk(121); BSS:tv2.dk(58); OpenEPG:TV2.dk(51)</t>
+          <t>EPGShare:TV.2.dk(115); BSS:tv2.dk(58); OpenEPG:TV 2.dk(57)</t>
         </is>
       </c>
     </row>
@@ -8445,7 +8429,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
@@ -8454,7 +8438,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.dk(121); BSS:tv2.dk(58); OpenEPG:TV2.dk(51)</t>
+          <t>EPGShare:TV.2.dk(115); BSS:tv2.dk(58); OpenEPG:TV 2.dk(57)</t>
         </is>
       </c>
     </row>
@@ -8491,7 +8475,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
@@ -8500,7 +8484,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Charlie.dk(105); BSS:tv2charlie.dk(50); OpenEPG:TV2 Charlie.dk(46)</t>
+          <t>EPGShare:TV.2.Charlie.dk(101); BSS:tv2charlie.dk(50); OpenEPG:TV 2 Charlie.dk(101)</t>
         </is>
       </c>
     </row>
@@ -8537,7 +8521,7 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
@@ -8546,7 +8530,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Charlie.dk(105); BSS:tv2charlie.dk(50); OpenEPG:TV2 Charlie.dk(46)</t>
+          <t>EPGShare:TV.2.Charlie.dk(101); BSS:tv2charlie.dk(50); OpenEPG:TV 2 Charlie.dk(101)</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8567,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
@@ -8592,7 +8576,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Charlie.dk(105); BSS:tv2charlie.dk(50); OpenEPG:TV2 Charlie.dk(46)</t>
+          <t>EPGShare:TV.2.Charlie.dk(101); BSS:tv2charlie.dk(50); OpenEPG:TV 2 Charlie.dk(101)</t>
         </is>
       </c>
     </row>
@@ -8629,7 +8613,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
@@ -8638,7 +8622,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Sport.dk(72); BSS:tv2sport.dk(35); OpenEPG:TV2 Sport.dk(30)</t>
+          <t>EPGShare:TV.2.Sport.dk(78); BSS:tv2sport.dk(35); OpenEPG:TV 2 Sport.dk(64)</t>
         </is>
       </c>
     </row>
@@ -8675,7 +8659,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
@@ -8684,7 +8668,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Sport.dk(72); BSS:tv2sport.dk(35); OpenEPG:TV2 Sport.dk(30)</t>
+          <t>EPGShare:TV.2.Sport.dk(78); BSS:tv2sport.dk(35); OpenEPG:TV 2 Sport.dk(64)</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8705,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
@@ -8730,7 +8714,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>EPGShare:TV.2.Sport.dk(72); BSS:tv2sport.dk(35); OpenEPG:TV2 Sport.dk(30)</t>
+          <t>EPGShare:TV.2.Sport.dk(78); BSS:tv2sport.dk(35); OpenEPG:TV 2 Sport.dk(64)</t>
         </is>
       </c>
     </row>
@@ -8767,7 +8751,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
@@ -8776,7 +8760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.MAX.dk(95); BSS:tv3max.dk(46); OpenEPG:tv3max.dk(52)</t>
+          <t>EPGShare:TV3.MAX.dk(82); BSS:tv3max.dk(46); OpenEPG:TV3 Max.dk(143)</t>
         </is>
       </c>
     </row>
@@ -8813,7 +8797,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
@@ -8822,7 +8806,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.MAX.dk(95); BSS:tv3max.dk(46); OpenEPG:tv3max.dk(52)</t>
+          <t>EPGShare:TV3.MAX.dk(82); BSS:tv3max.dk(46); OpenEPG:TV3 Max.dk(143)</t>
         </is>
       </c>
     </row>
@@ -8859,7 +8843,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
@@ -8868,7 +8852,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.MAX.dk(95); BSS:tv3max.dk(46); OpenEPG:tv3max.dk(52)</t>
+          <t>EPGShare:TV3.MAX.dk(82); BSS:tv3max.dk(46); OpenEPG:TV3 Max.dk(143)</t>
         </is>
       </c>
     </row>
@@ -8905,7 +8889,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
@@ -8914,7 +8898,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.Puls.dk(104); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
+          <t>EPGShare:TV3.Puls.dk(97); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8935,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
@@ -8960,7 +8944,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.Puls.dk(104); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
+          <t>EPGShare:TV3.Puls.dk(97); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8981,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
@@ -9006,7 +8990,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.Puls.dk(104); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
+          <t>EPGShare:TV3.Puls.dk(97); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
         </is>
       </c>
     </row>
@@ -9043,7 +9027,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
@@ -9052,7 +9036,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.SPORT.dk(68); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
+          <t>EPGShare:TV3.SPORT.dk(70); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
         </is>
       </c>
     </row>
@@ -9089,7 +9073,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
@@ -9098,7 +9082,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.SPORT.dk(68); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
+          <t>EPGShare:TV3.SPORT.dk(70); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
         </is>
       </c>
     </row>
@@ -9135,7 +9119,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
@@ -9144,7 +9128,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.SPORT.dk(68); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
+          <t>EPGShare:TV3.SPORT.dk(70); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
         </is>
       </c>
     </row>
@@ -9156,7 +9140,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -9176,7 +9160,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -9189,12 +9173,12 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
         </is>
       </c>
     </row>
@@ -9206,7 +9190,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -9226,7 +9210,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -9239,12 +9223,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
         </is>
       </c>
     </row>
@@ -9256,7 +9240,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -9276,345 +9260,361 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
+          <t>tv3.dk</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>TV3.dk</t>
+        </is>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>kendt alternativt kilde-ID</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>TV3+ DK [Denmark]</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
           <t>tv3plus.dk</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="H126" t="n">
-        <v>0</v>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="H127" t="n">
+        <v>175</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
         <is>
           <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>kendt alternativt kilde-ID</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>FHD</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>TV3+ FHD DK [Denmark]</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>tv3plus.dk</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="H128" t="n">
+        <v>175</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>kendt alternativt kilde-ID</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>TV3+ HD DK [Denmark]</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>tv3plus.dk</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="H129" t="n">
+        <v>175</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>V Series.dk</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>FHD</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>V Series FHD DK [Multi-Sub] [Denmark]</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>viasatseries.dk</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>viasatseries.dk</t>
+        </is>
+      </c>
+      <c r="H130" t="n">
+        <v>154</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>DA).dk, V Series Denmark (DK, V Series.dk, V series HD (T).dk, V.series.dk, Viasat Series.dk, viasatseries.dk</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>BSS:viasatseries.dk(75); OpenEPG:Viasat Series.dk(167)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>V Series.dk</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>V Series HD DK [Denmark]</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>viasatseries.dk</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>viasatseries.dk</t>
+        </is>
+      </c>
+      <c r="H131" t="n">
+        <v>154</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>DA).dk, V Series Denmark (DK, V Series.dk, V series HD (T).dk, V.series.dk, Viasat Series.dk, viasatseries.dk</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>BSS:viasatseries.dk(75); OpenEPG:Viasat Series.dk(167)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Viaplay Sport News.dk</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Viaplay Sport News HD DK [Denmark]</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>viaplaysportnews.dk</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>viaplaysportnews.dk</t>
+        </is>
+      </c>
+      <c r="H132" t="n">
+        <v>78</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Viaplay Sport News HD (D) (T).dk, Viaplay Sport News.dk, Viaplay.Sport.News.dk, viaplaysportnews.dk</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>EPGShare:Viaplay.Sport.News.dk(78); BSS:viaplaysportnews.dk(40); OpenEPG:Viaplay Sport News.dk(68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Viasat Family.dk</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
         <is>
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="H127" t="n">
-        <v>0</v>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>TV3 DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H128" t="n">
-        <v>180</v>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>FHD</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>TV3 FHD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H129" t="n">
-        <v>180</v>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>TV3 HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H130" t="n">
-        <v>180</v>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H131" t="n">
-        <v>180</v>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J131" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>FHD</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>TV3+ FHD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H132" t="n">
-        <v>180</v>
-      </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>TV3+ HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr"/>
+          <t>V Film Family DK [Multi-Sub] [Denmark]</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>viasatfamily.dk</t>
+        </is>
+      </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>TV3+.dk</t>
+          <t>viasatfamily.dk</t>
         </is>
       </c>
       <c r="H133" t="n">
-        <v>180</v>
+        <v>49</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr"/>
+          <t>viasatfamily.dk</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>BSS:viasatfamily.dk(24); OpenEPG:viasatfamily.dk(27)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -9625,40 +9625,40 @@
       <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
-          <t>V Series.dk</t>
+          <t>Viasat Family.dk</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>FHD</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>V Series FHD DK [Multi-Sub] [Denmark]</t>
+          <t>V Film Family HD DK [Denmark]</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>viasatseries.dk</t>
+          <t>viasatfamily.dk</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>viasatseries.dk</t>
+          <t>viasatfamily.dk</t>
         </is>
       </c>
       <c r="H134" t="n">
-        <v>145</v>
+        <v>49</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>DA).dk, V Series Denmark (DK, V Series.dk, V series HD (T).dk, V.series.dk, Viasat Series.dk, viasatseries.dk</t>
+          <t>viasatfamily.dk</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>BSS:viasatseries.dk(75); OpenEPG:viasatseries.dk(83)</t>
+          <t>BSS:viasatfamily.dk(24); OpenEPG:viasatfamily.dk(27)</t>
         </is>
       </c>
     </row>
@@ -9671,40 +9671,40 @@
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
-          <t>V Series.dk</t>
+          <t>Viasat Nature Nordic Denmark (DK,DA).dk</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>FHD</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>V Series HD DK [Denmark]</t>
+          <t>Viasat Nature FHD DK [Multi-Sub] [Denmark]</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>viasatseries.dk</t>
+          <t>viasatnature.dk</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>viasatseries.dk</t>
+          <t>viasatnature.dk</t>
         </is>
       </c>
       <c r="H135" t="n">
-        <v>145</v>
+        <v>91</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>DA).dk, V Series Denmark (DK, V Series.dk, V series HD (T).dk, V.series.dk, Viasat Series.dk, viasatseries.dk</t>
+          <t>DA).dk, Viasat Nature HD (T).dk, Viasat Nature Nordic Denmark (DK, Viasat Nature.dk, Viasat.Nature.dk, viasatnature.dk</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>BSS:viasatseries.dk(75); OpenEPG:viasatseries.dk(83)</t>
+          <t>EPGShare:Viasat.Nature.dk(91); BSS:viasatnature.dk(48); OpenEPG:Viasat Nature.dk(98)</t>
         </is>
       </c>
     </row>
@@ -9717,7 +9717,7 @@
       <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Viaplay Sport News.dk</t>
+          <t>Viasat Nature Nordic Denmark (DK,DA).dk</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -9727,219 +9727,35 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Viaplay Sport News HD DK [Denmark]</t>
+          <t>Viasat Nature HD DK [Denmark]</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>viaplaysportnews.dk</t>
+          <t>viasatnature.dk</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>viaplaysportnews.dk</t>
+          <t>viasatnature.dk</t>
         </is>
       </c>
       <c r="H136" t="n">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Viaplay Sport News HD (D) (T).dk, Viaplay Sport News.dk, Viaplay.Sport.News.dk, viaplaysportnews.dk</t>
+          <t>DA).dk, Viasat Nature HD (T).dk, Viasat Nature Nordic Denmark (DK, Viasat Nature.dk, Viasat.Nature.dk, viasatnature.dk</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>EPGShare:Viaplay.Sport.News.dk(77); BSS:viaplaysportnews.dk(40); OpenEPG:Viaplay Sport News.dk(68)</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr"/>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>Viasat Family.dk</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>V Film Family DK [Multi-Sub] [Denmark]</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>viasatfamily.dk</t>
-        </is>
-      </c>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t>viasatfamily.dk</t>
-        </is>
-      </c>
-      <c r="H137" t="n">
-        <v>49</v>
-      </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>viasatfamily.dk</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>BSS:viasatfamily.dk(24); OpenEPG:viasatfamily.dk(27)</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>Viasat Family.dk</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>V Film Family HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>viasatfamily.dk</t>
-        </is>
-      </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>viasatfamily.dk</t>
-        </is>
-      </c>
-      <c r="H138" t="n">
-        <v>49</v>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>viasatfamily.dk</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>BSS:viasatfamily.dk(24); OpenEPG:viasatfamily.dk(27)</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr"/>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Viasat Nature Nordic Denmark (DK,DA).dk</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>FHD</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Viasat Nature FHD DK [Multi-Sub] [Denmark]</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>viasatnature.dk</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>viasatnature.dk</t>
-        </is>
-      </c>
-      <c r="H139" t="n">
-        <v>92</v>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>DA).dk, Viasat Nature HD (T).dk, Viasat Nature Nordic Denmark (DK, Viasat Nature.dk, Viasat.Nature.dk, viasatnature.dk</t>
-        </is>
-      </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t>EPGShare:Viasat.Nature.dk(92); BSS:viasatnature.dk(48); OpenEPG:Viasat Nature.dk(98)</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>Viasat Nature Nordic Denmark (DK,DA).dk</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Viasat Nature HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>viasatnature.dk</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>viasatnature.dk</t>
-        </is>
-      </c>
-      <c r="H140" t="n">
-        <v>92</v>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>DA).dk, Viasat Nature HD (T).dk, Viasat Nature Nordic Denmark (DK, Viasat Nature.dk, Viasat.Nature.dk, viasatnature.dk</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>EPGShare:Viasat.Nature.dk(92); BSS:viasatnature.dk(48); OpenEPG:Viasat Nature.dk(98)</t>
+          <t>EPGShare:Viasat.Nature.dk(91); BSS:viasatnature.dk(48); OpenEPG:Viasat Nature.dk(98)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J140"/>
+  <autoFilter ref="A1:J136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9950,11 +9766,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
@@ -9962,7 +9778,7 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10063,7 +9879,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10083,7 +9899,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -10096,12 +9912,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
         </is>
       </c>
     </row>
@@ -10113,7 +9929,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -10133,7 +9949,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -10146,12 +9962,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
         </is>
       </c>
     </row>
@@ -10163,7 +9979,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -10183,7 +9999,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -10196,335 +10012,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>TV3 DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>180</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>FHD</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>TV3 FHD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>180</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>TV3 HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>180</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>180</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>FHD</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>TV3+ FHD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>180</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>TV3+ HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>180</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10535,11 +10033,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
@@ -10635,7 +10133,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -10644,7 +10142,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.MAX.dk(95); BSS:tv3max.dk(46); OpenEPG:tv3max.dk(52)</t>
+          <t>EPGShare:TV3.MAX.dk(82); BSS:tv3max.dk(46); OpenEPG:TV3 Max.dk(143)</t>
         </is>
       </c>
     </row>
@@ -10681,7 +10179,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -10690,7 +10188,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.MAX.dk(95); BSS:tv3max.dk(46); OpenEPG:tv3max.dk(52)</t>
+          <t>EPGShare:TV3.MAX.dk(82); BSS:tv3max.dk(46); OpenEPG:TV3 Max.dk(143)</t>
         </is>
       </c>
     </row>
@@ -10727,7 +10225,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -10736,7 +10234,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.MAX.dk(95); BSS:tv3max.dk(46); OpenEPG:tv3max.dk(52)</t>
+          <t>EPGShare:TV3.MAX.dk(82); BSS:tv3max.dk(46); OpenEPG:TV3 Max.dk(143)</t>
         </is>
       </c>
     </row>
@@ -10773,7 +10271,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -10782,7 +10280,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.Puls.dk(104); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
+          <t>EPGShare:TV3.Puls.dk(97); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
         </is>
       </c>
     </row>
@@ -10819,7 +10317,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -10828,7 +10326,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.Puls.dk(104); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
+          <t>EPGShare:TV3.Puls.dk(97); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
         </is>
       </c>
     </row>
@@ -10865,7 +10363,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -10874,7 +10372,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.Puls.dk(104); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
+          <t>EPGShare:TV3.Puls.dk(97); BSS:tv3puls.dk(46); OpenEPG:TV3 Puls.dk(135)</t>
         </is>
       </c>
     </row>
@@ -10911,7 +10409,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -10920,7 +10418,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.SPORT.dk(68); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
+          <t>EPGShare:TV3.SPORT.dk(70); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
         </is>
       </c>
     </row>
@@ -10957,7 +10455,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -10966,7 +10464,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.SPORT.dk(68); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
+          <t>EPGShare:TV3.SPORT.dk(70); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
         </is>
       </c>
     </row>
@@ -11003,7 +10501,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -11012,7 +10510,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>EPGShare:TV3.SPORT.dk(68); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
+          <t>EPGShare:TV3.SPORT.dk(70); BSS:tv3sport.dk(27); OpenEPG:TV3 Sport.dk(94)</t>
         </is>
       </c>
     </row>
@@ -11024,7 +10522,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -11044,7 +10542,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -11057,12 +10555,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
         </is>
       </c>
     </row>
@@ -11074,7 +10572,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -11094,7 +10592,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>tv3plus.dk</t>
+          <t>tv3.dk</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -11107,12 +10605,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
         </is>
       </c>
     </row>
@@ -11124,7 +10622,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>kendt alternativt kilde-ID, output-ID har 0 programmer</t>
+          <t>output-ID har 0 programmer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -11144,79 +10642,87 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>tv3.dk</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TV3.dk</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3.dk, tv3.dk</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>EPGShare:TV3.dk(82); BSS:tv3.dk(43); OpenEPG:tv3.dk(43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>kendt alternativt kilde-ID</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TV3+ DK [Denmark]</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>tv3plus.dk</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>TV3+.dk</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>175</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>TV3.dk</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3 Denmark (DK, TV3 HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
+          <t>kendt alternativt kilde-ID</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -11226,12 +10732,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>FHD</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TV3 DK [Denmark]</t>
+          <t>TV3+ FHD DK [Denmark]</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -11245,11 +10751,11 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -11259,14 +10765,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
+          <t>kendt alternativt kilde-ID</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -11276,12 +10782,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>FHD</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TV3 FHD DK [Denmark]</t>
+          <t>TV3+ HD DK [Denmark]</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -11295,11 +10801,11 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
+          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, tv3plus.dk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -11308,184 +10814,8 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>FORKERT KANAL</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>TV3+-gruppen indeholder en TV3 stream</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>TV3 HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>180</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>BSS:tv3plus.dk(42); OpenEPG:tv3plus.dk(43)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>TV3+ DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>180</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>FHD</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>TV3+ FHD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>180</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>MANGLER TVG-ID</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Streamen har intet tvg-id</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>TV3+ HD DK [Denmark]</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>TV3+.dk</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>180</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>DA).dk, TV3+ Denmark (DK, TV3+ HD (D) (T).dk, TV3+.dk, TV3.dk, tv3.dk, tv3plus.dk</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J20"/>
+  <autoFilter ref="A1:J16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>